<commit_message>
Document the self-hosted platform beside the Supabase configuration (2126)
Row 5.10 of the stage 5 plan, the half that can be written honestly
before the Supabase project is gone. docs/deployment.md gains a section
on the platform: the three SUPABASE_* variables keep their names and
meaning and only their values move, the modules and their READMEs, the
two gating variables, and how database setup runs through the dbtools
task. first-apply.md gains the stage 5 apply sequence. architecture.md's
decision 4 records its own supersession and the cost table carries the
platform's rows. The docs index lists the three stage 5 runbooks.

The pass that removes the Supabase paragraphs waits for Stage 5, Task 6.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q7XSyAdd4z5XDWLFBwTa8L
</commit_message>
<xml_diff>
--- a/docs/delivery-plan/v2/delivery-status.xlsx
+++ b/docs/delivery-plan/v2/delivery-status.xlsx
@@ -10821,7 +10821,7 @@
       </c>
       <c r="F123" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 1 in progress, 1 to do.</t>
+          <t>Rolled up from 2 children: 2 in progress.</t>
         </is>
       </c>
       <c r="G123" s="20" t="inlineStr">
@@ -10958,14 +10958,14 @@
           <t>Update the documentation</t>
         </is>
       </c>
-      <c r="E125" s="25" t="inlineStr">
-        <is>
-          <t>To do</t>
+      <c r="E125" s="22" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F125" s="23" t="inlineStr">
         <is>
-          <t>Stage 5, added 17 September 2026.</t>
+          <t>The platform is documented beside Supabase (plan row 5.10); the pass that removes the Supabase paragraphs waits for Stage 5, Task 6.</t>
         </is>
       </c>
       <c r="G125" s="20" t="inlineStr">
@@ -12952,7 +12952,7 @@
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 1 in progress, 1 to do.</t>
+          <t>Rolled up from 2 children: 2 in progress.</t>
         </is>
       </c>
       <c r="F44" s="20" t="inlineStr">
@@ -12992,14 +12992,14 @@
           <t>Update the documentation</t>
         </is>
       </c>
-      <c r="D45" s="25" t="inlineStr">
-        <is>
-          <t>To do</t>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>Stage 5, added 17 September 2026.</t>
+          <t>The platform is documented beside Supabase (plan row 5.10); the pass that removes the Supabase paragraphs waits for Stage 5, Task 6.</t>
         </is>
       </c>
       <c r="F45" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Size the first upstream sync from a rehearsed merge (2009)
The dry run ticket 2009 asked for was never done while a conflict was
impossible. Rehearsed on a full-history checkout on 17 September 2026:
36 upstream commits since the seed, 49 conflicted files, four of them
collisions with positions the fork took deliberately (a shared contracts
package against the frontend boundary, the SheetJS CDN against the
pinned republish, the icon rewrite against the brand mark, and the route
refactor against the fork's audit and Express 5 edits), and 40 files
that would reintroduce the upstream name. Written into
docs/upstream-sync.md with a recommendation to run it as its own sprint.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q7XSyAdd4z5XDWLFBwTa8L
</commit_message>
<xml_diff>
--- a/docs/delivery-plan/v2/delivery-status.xlsx
+++ b/docs/delivery-plan/v2/delivery-status.xlsx
@@ -62,13 +62,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00434343"/>
+      <color rgb="00990000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00990000"/>
+      <color rgb="00434343"/>
       <sz val="10"/>
     </font>
     <font>
@@ -126,12 +126,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8EAED"/>
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="00E8EAED"/>
       </patternFill>
     </fill>
     <fill>
@@ -205,7 +205,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -214,7 +214,7 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2730,14 +2730,14 @@
           <t>Run a first upstream merge as a dry run</t>
         </is>
       </c>
-      <c r="E10" s="25" t="inlineStr">
-        <is>
-          <t>To do</t>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>Never performed in this fork; the "upstream" merges in history are inherited. Value decays as the fork diverges.</t>
+          <t>Rehearsed in a scratch worktree on 17 September 2026 and sized in docs/upstream-sync.md ("The first sync, sized"): 49 conflicts, four of them decisions against fork positions, plus 40 files to debrand. Recommended as its own sprint.</t>
         </is>
       </c>
       <c r="G10" s="20" t="inlineStr">
@@ -2942,7 +2942,7 @@
           <t>Replace xlsx with exceljs in spreadsheet.ts</t>
         </is>
       </c>
-      <c r="E13" s="26" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>Won't do</t>
         </is>
@@ -3086,7 +3086,7 @@
           <t>Take ownership of the workflow catalogue</t>
         </is>
       </c>
-      <c r="E15" s="25" t="inlineStr">
+      <c r="E15" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -3158,7 +3158,7 @@
           <t>Fork mike-workflows and repoint the sync</t>
         </is>
       </c>
-      <c r="E16" s="25" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -3230,7 +3230,7 @@
           <t>Verify catalogue sync end to end</t>
         </is>
       </c>
-      <c r="E17" s="25" t="inlineStr">
+      <c r="E17" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -3730,7 +3730,7 @@
           <t>Disable the Word add-in workflow while the add-in is deferred</t>
         </is>
       </c>
-      <c r="E24" s="26" t="inlineStr">
+      <c r="E24" s="25" t="inlineStr">
         <is>
           <t>Won't do</t>
         </is>
@@ -9166,7 +9166,7 @@
           <t>Address what the load test surfaces</t>
         </is>
       </c>
-      <c r="E100" s="25" t="inlineStr">
+      <c r="E100" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -9378,7 +9378,7 @@
           <t>Run the full suite against production configuration</t>
         </is>
       </c>
-      <c r="E103" s="25" t="inlineStr">
+      <c r="E103" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -9738,7 +9738,7 @@
           <t>Post-launch monitoring window</t>
         </is>
       </c>
-      <c r="E108" s="25" t="inlineStr">
+      <c r="E108" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -11253,7 +11253,7 @@
           <t>Take ownership of the workflow catalogue</t>
         </is>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -11300,7 +11300,7 @@
           <t>Fork mike-workflows and repoint the sync</t>
         </is>
       </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="D9" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -11347,14 +11347,14 @@
           <t>Run a first upstream merge as a dry run</t>
         </is>
       </c>
-      <c r="D10" s="25" t="inlineStr">
-        <is>
-          <t>To do</t>
+      <c r="D10" s="22" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>Never performed in this fork; the "upstream" merges in history are inherited. Value decays as the fork diverges.</t>
+          <t>Rehearsed in a scratch worktree on 17 September 2026 and sized in docs/upstream-sync.md ("The first sync, sized"): 49 conflicts, four of them decisions against fork positions, plus 40 files to debrand. Recommended as its own sprint.</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
@@ -11394,7 +11394,7 @@
           <t>Verify catalogue sync end to end</t>
         </is>
       </c>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -12099,7 +12099,7 @@
           <t>Run the full suite against production configuration</t>
         </is>
       </c>
-      <c r="D26" s="25" t="inlineStr">
+      <c r="D26" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -12334,7 +12334,7 @@
           <t>Post-launch monitoring window</t>
         </is>
       </c>
-      <c r="D31" s="25" t="inlineStr">
+      <c r="D31" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -12522,7 +12522,7 @@
           <t>Address what the load test surfaces</t>
         </is>
       </c>
-      <c r="D35" s="25" t="inlineStr">
+      <c r="D35" s="26" t="inlineStr">
         <is>
           <t>To do</t>
         </is>

</xml_diff>

<commit_message>
Answer the catalogue licence question ticket 2015 raises
The workflow catalogue repository is MIT at ce62e6a, with a provenance
policy for adapted packs. That clears the licence check the ticket asks
for before the fork; the fork itself needs an account only the operator
controls, and after it the repoint is two tfvars values and an apply.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q7XSyAdd4z5XDWLFBwTa8L
</commit_message>
<xml_diff>
--- a/docs/delivery-plan/v2/delivery-status.xlsx
+++ b/docs/delivery-plan/v2/delivery-status.xlsx
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>Inherited from parent 2014 (to do).</t>
+          <t>Licence checked 17 September 2026: the catalogue repository is MIT (outstanding.md). The fork itself needs an account only the operator controls; after it, two tfvars values and an apply.</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>Inherited from parent 2014 (to do).</t>
+          <t>Licence checked 17 September 2026: the catalogue repository is MIT (outstanding.md). The fork itself needs an account only the operator controls; after it, two tfvars values and an apply.</t>
         </is>
       </c>
       <c r="F9" s="20" t="inlineStr">

</xml_diff>

<commit_message>
F0-1: Architecture decision 7 — fold-in, not a Juralio HTTP seam (#117)
* Record architecture decision 7: fold-in, not a Juralio HTTP seam.

Cancel tickets 2066–2069. Keep boundary CI (2070). Cite Matter
Management as specification-only prior art in NOTICE. ISMS production
scope is this origin only.

Co-authored-by: frasermatcham <frasermatcham@gmail.com>

* Keep 2070 Done and use a workbook-valid Superseded status.

The architecture table cancelled 2066–2070, which would have retired
boundary CI. Only the HTTP-seam tickets 2066–2069 are cancelled.
status.csv now uses the existing Superseded token so the workbook
script can colour and count those rows.

Co-authored-by: frasermatcham <frasermatcham@gmail.com>

---------

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/delivery-plan/v2/delivery-status.xlsx
+++ b/docs/delivery-plan/v2/delivery-status.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tickets'!$A$1:$N$125</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outstanding'!$A$4:$I$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outstanding'!$A$4:$I$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -74,12 +74,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00674EA7"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00434343"/>
       <sz val="10"/>
     </font>
@@ -100,6 +94,12 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00674EA7"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -136,12 +136,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
+        <fgColor rgb="00E8EAED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8EAED"/>
+        <fgColor rgb="00D9D2E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -171,11 +171,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -205,10 +205,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,7 +217,7 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -242,9 +242,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1972,7 +1969,7 @@
       </c>
       <c r="B55" s="13" t="inlineStr">
         <is>
-          <t>Replaced by the stage 5 move off Supabase; the work no longer applies.</t>
+          <t>Replaced by a later decision: stage 5 (off Supabase) or architecture decision 7 (fold-in, not a Juralio HTTP seam).</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2009,7 @@
     <row r="61" ht="26" customHeight="1">
       <c r="A61" s="19" t="inlineStr">
         <is>
-          <t>- The twelve tickets with no marker are resolved explicitly by the plan's ticket disposition table (2023 won't do; 2029-2031 done; 2038-2041 superseded by stage 5; 2066-2069 deferred).</t>
+          <t>- The twelve tickets with no marker are resolved explicitly by the plan's ticket disposition table (2023 won't do; 2029-2031 done; 2038-2041 superseded by stage 5; 2066-2069 cancelled by architecture decision 7).</t>
         </is>
       </c>
     </row>
@@ -6734,14 +6731,14 @@
           <t>Integration with the Juralio platform</t>
         </is>
       </c>
-      <c r="E66" s="22" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E66" s="26" t="inlineStr">
+        <is>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="F66" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 1 done, 1 deferred.</t>
+          <t>Epic kept as the licence-boundary record. Child 2070 (boundary CI) shipped and stays Done. HTTP seam children 2066–2069 cancelled — architecture decision 7.</t>
         </is>
       </c>
       <c r="G66" s="20" t="inlineStr">
@@ -6806,14 +6803,14 @@
           <t>Build the HTTP client seam in Juralio</t>
         </is>
       </c>
-      <c r="E67" s="27" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E67" s="26" t="inlineStr">
+        <is>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="F67" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 3 children: 3 deferred.</t>
+          <t>HTTP client seam in Juralio cancelled. Reimplement matter features in this origin (architecture decision 7).</t>
         </is>
       </c>
       <c r="G67" s="20" t="inlineStr">
@@ -6878,9 +6875,9 @@
           <t>Write Juralio's proxy to the workflow service</t>
         </is>
       </c>
-      <c r="E68" s="27" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E68" s="26" t="inlineStr">
+        <is>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="F68" s="23" t="inlineStr">
@@ -6950,9 +6947,9 @@
           <t>Re-declare the API types on the Juralio side</t>
         </is>
       </c>
-      <c r="E69" s="27" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E69" s="26" t="inlineStr">
+        <is>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="F69" s="23" t="inlineStr">
@@ -7022,9 +7019,9 @@
           <t>Map identity and sessions between the two systems</t>
         </is>
       </c>
-      <c r="E70" s="27" t="inlineStr">
-        <is>
-          <t>Deferred</t>
+      <c r="E70" s="26" t="inlineStr">
+        <is>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="F70" s="23" t="inlineStr">
@@ -7101,7 +7098,7 @@
       </c>
       <c r="F71" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 1 child: 1 done.</t>
+          <t>Boundary CI shipped (`npm run boundary`). Seam itself superseded: fold-in (architecture decision 7). Keep the CI.</t>
         </is>
       </c>
       <c r="G71" s="20" t="inlineStr">
@@ -9166,7 +9163,7 @@
           <t>Address what the load test surfaces</t>
         </is>
       </c>
-      <c r="E100" s="28" t="inlineStr">
+      <c r="E100" s="27" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -9378,7 +9375,7 @@
           <t>Run the full suite against production configuration</t>
         </is>
       </c>
-      <c r="E103" s="28" t="inlineStr">
+      <c r="E103" s="27" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -11021,7 +11018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11616,17 +11613,17 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>2065</t>
+          <t>2094</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>Integration with the Juralio platform</t>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Backup, restore and disaster recovery</t>
         </is>
       </c>
       <c r="D16" s="22" t="inlineStr">
@@ -11636,22 +11633,22 @@
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 1 done, 1 deferred.</t>
+          <t>Rolled up from 2 children: 1 done, 1 in progress.</t>
         </is>
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Phase 2 - Infrastructure</t>
+          <t>Phase 3 - Production Ready</t>
         </is>
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 6</t>
         </is>
       </c>
       <c r="H16" s="20" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="I16" s="20" t="inlineStr">
@@ -11663,17 +11660,17 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>2094</t>
+          <t>2095</t>
         </is>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Sub-task</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Backup, restore and disaster recovery</t>
+          <t>Configure automated backups and prove a restore</t>
         </is>
       </c>
       <c r="D17" s="22" t="inlineStr">
@@ -11683,7 +11680,7 @@
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 1 done, 1 in progress.</t>
+          <t>Drilled 18 September 2026, partial. Documents passed: a document deleted from production was recovered from the backup bucket by version id, size and ETag matching, and live/backup are identical across all 8 objects with every one ReplicationStatus COMPLETED. Database could not be attempted: the Supabase org is on the Free plan, which has no accessible daily backups, and no self-managed dump exists. Stays open until the database has a backup and the application can be run against restored data.</t>
         </is>
       </c>
       <c r="F17" s="20" t="inlineStr">
@@ -11710,17 +11707,17 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2095</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Sub-task</t>
-        </is>
-      </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>Configure automated backups and prove a restore</t>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Launch</t>
         </is>
       </c>
       <c r="D18" s="22" t="inlineStr">
@@ -11730,7 +11727,7 @@
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>Drilled 18 September 2026, partial. Documents passed: a document deleted from production was recovered from the backup bucket by version id, size and ETag matching, and live/backup are identical across all 8 objects with every one ReplicationStatus COMPLETED. Database could not be attempted: the Supabase org is on the Free plan, which has no accessible daily backups, and no self-managed dump exists. Stays open until the database has a backup and the application can be run against restored data.</t>
+          <t>Rolled up from 2 children: 2 in progress.</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
@@ -11745,7 +11742,7 @@
       </c>
       <c r="H18" s="20" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="I18" s="20" t="inlineStr">
@@ -11757,17 +11754,17 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2101</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>Launch</t>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Pre-launch verification</t>
         </is>
       </c>
       <c r="D19" s="22" t="inlineStr">
@@ -11777,7 +11774,7 @@
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 2 in progress.</t>
+          <t>Rolled up from 3 children: 2 in progress, 1 to do.</t>
         </is>
       </c>
       <c r="F19" s="20" t="inlineStr">
@@ -11804,27 +11801,27 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2101</t>
+          <t>2102</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Sub-task</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>Pre-launch verification</t>
-        </is>
-      </c>
-      <c r="D20" s="22" t="inlineStr">
-        <is>
-          <t>In progress</t>
+          <t>Run the full suite against production configuration</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>To do</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 3 children: 2 in progress, 1 to do.</t>
+          <t>From the delivery plan row that cites it.</t>
         </is>
       </c>
       <c r="F20" s="20" t="inlineStr">
@@ -11851,7 +11848,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t>2102</t>
+          <t>2104</t>
         </is>
       </c>
       <c r="B21" s="20" t="inlineStr">
@@ -11861,17 +11858,17 @@
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Run the full suite against production configuration</t>
-        </is>
-      </c>
-      <c r="D21" s="28" t="inlineStr">
-        <is>
-          <t>To do</t>
+          <t>Security review of the combined deployment</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
         <is>
-          <t>From the delivery plan row that cites it.</t>
+          <t>This repository half done: 3 findings, all fixed. Juralio side and the seam from its end outstanding.</t>
         </is>
       </c>
       <c r="F21" s="20" t="inlineStr">
@@ -11898,17 +11895,17 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2104</t>
+          <t>2105</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Sub-task</t>
+          <t>Story</t>
         </is>
       </c>
       <c r="C22" s="23" t="inlineStr">
         <is>
-          <t>Security review of the combined deployment</t>
+          <t>Go live</t>
         </is>
       </c>
       <c r="D22" s="22" t="inlineStr">
@@ -11918,7 +11915,7 @@
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>This repository half done: 3 findings, all fixed. Juralio side and the seam from its end outstanding.</t>
+          <t>Rolled up from 2 children: 1 in progress, 1 to do.</t>
         </is>
       </c>
       <c r="F22" s="20" t="inlineStr">
@@ -11945,17 +11942,17 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t>2105</t>
+          <t>2107</t>
         </is>
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Sub-task</t>
         </is>
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>Go live</t>
+          <t>Post-launch monitoring window</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
@@ -11965,7 +11962,7 @@
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 1 in progress, 1 to do.</t>
+          <t>Alerting proven working 18 September 2026: both SNS alert topics had zero subscriptions, so all 16 alarms fired into silence. Subscribed and confirmed, and a test publish to each topic was confirmed received. The subscriptions are account state, not Terraform: alert_email is now documented in terraform.tfvars.example and the module README carries the import commands that adopt the existing pair instead of duplicating them. Remaining: the monitoring window itself.</t>
         </is>
       </c>
       <c r="F23" s="20" t="inlineStr">
@@ -11992,17 +11989,17 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
-          <t>2107</t>
+          <t>2093</t>
         </is>
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Sub-task</t>
-        </is>
-      </c>
-      <c r="C24" s="23" t="inlineStr">
-        <is>
-          <t>Post-launch monitoring window</t>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>Operational readiness</t>
         </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
@@ -12012,7 +12009,7 @@
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>Alerting proven working 18 September 2026: both SNS alert topics had zero subscriptions, so all 16 alarms fired into silence. Subscribed and confirmed, and a test publish to each topic was confirmed received. The subscriptions are account state, not Terraform: alert_email is now documented in terraform.tfvars.example and the module README carries the import commands that adopt the existing pair instead of duplicating them. Remaining: the monitoring window itself.</t>
+          <t>Rolled up from 2 children: 2 in progress.</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
@@ -12027,29 +12024,29 @@
       </c>
       <c r="H24" s="20" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="I24" s="20" t="inlineStr">
         <is>
-          <t>Highest</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>2093</t>
+          <t>2097</t>
         </is>
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>Operational readiness</t>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Performance and resilience</t>
         </is>
       </c>
       <c r="D25" s="22" t="inlineStr">
@@ -12059,7 +12056,7 @@
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 2 in progress.</t>
+          <t>Rolled up from 2 children: 1 in progress, 1 to do.</t>
         </is>
       </c>
       <c r="F25" s="20" t="inlineStr">
@@ -12074,29 +12071,29 @@
       </c>
       <c r="H25" s="20" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="I25" s="20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
-          <t>2097</t>
+          <t>2098</t>
         </is>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Sub-task</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>Performance and resilience</t>
+          <t>Run the k6 SSE load scenario against staging</t>
         </is>
       </c>
       <c r="D26" s="22" t="inlineStr">
@@ -12106,7 +12103,7 @@
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 1 in progress, 1 to do.</t>
+          <t>Blocked on Task 3 (2020): without a provider key the SSE scenario measures how fast the service fails. Also needs a LOADTEST_AUTH_TOKEN and a decision on which stack to point at, since every iteration writes a real chat row and spends real tokens.</t>
         </is>
       </c>
       <c r="F26" s="20" t="inlineStr">
@@ -12133,7 +12130,7 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>2098</t>
+          <t>2099</t>
         </is>
       </c>
       <c r="B27" s="20" t="inlineStr">
@@ -12143,17 +12140,17 @@
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>Run the k6 SSE load scenario against staging</t>
-        </is>
-      </c>
-      <c r="D27" s="22" t="inlineStr">
-        <is>
-          <t>In progress</t>
+          <t>Address what the load test surfaces</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>To do</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>Blocked on Task 3 (2020): without a provider key the SSE scenario measures how fast the service fails. Also needs a LOADTEST_AUTH_TOKEN and a decision on which stack to point at, since every iteration writes a real chat row and spends real tokens.</t>
+          <t>From the delivery plan row that cites it.</t>
         </is>
       </c>
       <c r="F27" s="20" t="inlineStr">
@@ -12180,64 +12177,64 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2099</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Sub-task</t>
-        </is>
-      </c>
-      <c r="C28" s="23" t="inlineStr">
-        <is>
-          <t>Address what the load test surfaces</t>
-        </is>
-      </c>
-      <c r="D28" s="28" t="inlineStr">
-        <is>
-          <t>To do</t>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>Run the platform services on AWS instead of Supabase</t>
+        </is>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>From the delivery plan row that cites it.</t>
+          <t>Rolled up from 6 children: 1 done, 5 in progress.</t>
         </is>
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Phase 3 - Production Ready</t>
+          <t>Phase 4 - Self-hosted platform</t>
         </is>
       </c>
       <c r="G28" s="20" t="inlineStr">
         <is>
-          <t>Sprint 6</t>
+          <t>Sprint 7</t>
         </is>
       </c>
       <c r="H28" s="20" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="I28" s="20" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Highest</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>Run the platform services on AWS instead of Supabase</t>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>PostgREST as an ECS service</t>
         </is>
       </c>
       <c r="D29" s="22" t="inlineStr">
@@ -12247,7 +12244,7 @@
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 6 children: 1 done, 5 in progress.</t>
+          <t>Rolled up from 1 child: 1 done. Closes when the backend's queries succeed against the self-hosted endpoint after cutover.</t>
         </is>
       </c>
       <c r="F29" s="20" t="inlineStr">
@@ -12274,7 +12271,7 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>2116</t>
         </is>
       </c>
       <c r="B30" s="20" t="inlineStr">
@@ -12284,7 +12281,7 @@
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>PostgREST as an ECS service</t>
+          <t>GoTrue as an ECS service</t>
         </is>
       </c>
       <c r="D30" s="22" t="inlineStr">
@@ -12294,7 +12291,7 @@
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 1 child: 1 done. Closes when the backend's queries succeed against the self-hosted endpoint after cutover.</t>
+          <t>Rolled up from 3 children: 1 done, 2 in progress.</t>
         </is>
       </c>
       <c r="F30" s="20" t="inlineStr">
@@ -12321,7 +12318,7 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>2116</t>
+          <t>2120</t>
         </is>
       </c>
       <c r="B31" s="20" t="inlineStr">
@@ -12331,7 +12328,7 @@
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>GoTrue as an ECS service</t>
+          <t>Own the JWT secret and the API keys</t>
         </is>
       </c>
       <c r="D31" s="22" t="inlineStr">
@@ -12341,7 +12338,7 @@
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 3 children: 1 done, 2 in progress.</t>
+          <t>Rolled up from 1 child: 1 done. Closes when the runbook has been walked once against the applied footprint.</t>
         </is>
       </c>
       <c r="F31" s="20" t="inlineStr">
@@ -12368,7 +12365,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>2120</t>
+          <t>2122</t>
         </is>
       </c>
       <c r="B32" s="20" t="inlineStr">
@@ -12378,7 +12375,7 @@
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Own the JWT secret and the API keys</t>
+          <t>Routing and configuration cutover</t>
         </is>
       </c>
       <c r="D32" s="22" t="inlineStr">
@@ -12388,7 +12385,7 @@
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 1 child: 1 done. Closes when the runbook has been walked once against the applied footprint.</t>
+          <t>Rolled up from 1 child: 1 done. The platform_serves_backend switch exists; closes at the cutover.</t>
         </is>
       </c>
       <c r="F32" s="20" t="inlineStr">
@@ -12415,17 +12412,17 @@
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>2122</t>
+          <t>2125</t>
         </is>
       </c>
       <c r="B33" s="20" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Sub-task</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>Routing and configuration cutover</t>
+          <t>Rehearse the cutover and the rollback</t>
         </is>
       </c>
       <c r="D33" s="22" t="inlineStr">
@@ -12435,7 +12432,7 @@
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 1 child: 1 done. The platform_serves_backend switch exists; closes at the cutover.</t>
+          <t>Procedure written (docs/runbooks/platform-cutover.md) and the smoke test extended; the rehearsal itself needs the applied platform and Stage 5, Tasks 1 to 4.</t>
         </is>
       </c>
       <c r="F33" s="20" t="inlineStr">
@@ -12462,7 +12459,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>2125</t>
+          <t>2118</t>
         </is>
       </c>
       <c r="B34" s="20" t="inlineStr">
@@ -12472,7 +12469,7 @@
       </c>
       <c r="C34" s="23" t="inlineStr">
         <is>
-          <t>Rehearse the cutover and the rollback</t>
+          <t>Auth email through SES</t>
         </is>
       </c>
       <c r="D34" s="22" t="inlineStr">
@@ -12482,7 +12479,7 @@
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>Procedure written (docs/runbooks/platform-cutover.md) and the smoke test extended; the rehearsal itself needs the applied platform and Stage 5, Tasks 1 to 4.</t>
+          <t>Wired to the email module's SES credential (plan row 5.5); the deliverability check needs the running service.</t>
         </is>
       </c>
       <c r="F34" s="20" t="inlineStr">
@@ -12502,14 +12499,14 @@
       </c>
       <c r="I34" s="20" t="inlineStr">
         <is>
-          <t>Highest</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>2118</t>
+          <t>2119</t>
         </is>
       </c>
       <c r="B35" s="20" t="inlineStr">
@@ -12519,7 +12516,7 @@
       </c>
       <c r="C35" s="23" t="inlineStr">
         <is>
-          <t>Auth email through SES</t>
+          <t>Carry the Google OAuth provider across</t>
         </is>
       </c>
       <c r="D35" s="22" t="inlineStr">
@@ -12529,7 +12526,7 @@
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>Wired to the email module's SES credential (plan row 5.5); the deliverability check needs the running service.</t>
+          <t>Provider, secret container and redirect URI in place (plan row 5.6); the operator adds the URI and writes the client (Stage 5, Task 3).</t>
         </is>
       </c>
       <c r="F35" s="20" t="inlineStr">
@@ -12556,17 +12553,17 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>2119</t>
+          <t>2124</t>
         </is>
       </c>
       <c r="B36" s="20" t="inlineStr">
         <is>
-          <t>Sub-task</t>
+          <t>Story</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
         <is>
-          <t>Carry the Google OAuth provider across</t>
+          <t>Cutover and decommission</t>
         </is>
       </c>
       <c r="D36" s="22" t="inlineStr">
@@ -12576,7 +12573,7 @@
       </c>
       <c r="E36" s="23" t="inlineStr">
         <is>
-          <t>Provider, secret container and redirect URI in place (plan row 5.6); the operator adds the URI and writes the client (Stage 5, Task 3).</t>
+          <t>Rolled up from 2 children: 2 in progress.</t>
         </is>
       </c>
       <c r="F36" s="20" t="inlineStr">
@@ -12591,7 +12588,7 @@
       </c>
       <c r="H36" s="20" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="I36" s="20" t="inlineStr">
@@ -12603,17 +12600,17 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>2124</t>
+          <t>2126</t>
         </is>
       </c>
       <c r="B37" s="20" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Sub-task</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>Cutover and decommission</t>
+          <t>Update the documentation</t>
         </is>
       </c>
       <c r="D37" s="22" t="inlineStr">
@@ -12623,7 +12620,7 @@
       </c>
       <c r="E37" s="23" t="inlineStr">
         <is>
-          <t>Rolled up from 2 children: 2 in progress.</t>
+          <t>The platform is documented beside Supabase (plan row 5.10); the pass that removes the Supabase paragraphs waits for Stage 5, Task 6.</t>
         </is>
       </c>
       <c r="F37" s="20" t="inlineStr">
@@ -12643,77 +12640,30 @@
       </c>
       <c r="I37" s="20" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t>2126</t>
-        </is>
-      </c>
-      <c r="B38" s="20" t="inlineStr">
-        <is>
-          <t>Sub-task</t>
-        </is>
-      </c>
-      <c r="C38" s="23" t="inlineStr">
-        <is>
-          <t>Update the documentation</t>
-        </is>
-      </c>
-      <c r="D38" s="22" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="E38" s="23" t="inlineStr">
-        <is>
-          <t>The platform is documented beside Supabase (plan row 5.10); the pass that removes the Supabase paragraphs waits for Stage 5, Task 6.</t>
-        </is>
-      </c>
-      <c r="F38" s="20" t="inlineStr">
-        <is>
-          <t>Phase 4 - Self-hosted platform</t>
-        </is>
-      </c>
-      <c r="G38" s="20" t="inlineStr">
-        <is>
-          <t>Sprint 7</t>
-        </is>
-      </c>
-      <c r="H38" s="20" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="I38" s="20" t="inlineStr">
-        <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Open tickets</t>
+        </is>
+      </c>
+      <c r="B39" s="7">
+        <f>COUNTIF(Tickets!$E$2:$E$125,"In progress")+COUNTIF(Tickets!$E$2:$E$125,"To do")</f>
+        <v/>
+      </c>
+    </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Open tickets</t>
-        </is>
-      </c>
-      <c r="B40" s="7">
-        <f>COUNTIF(Tickets!$E$2:$E$125,"In progress")+COUNTIF(Tickets!$E$2:$E$125,"To do")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>The rows are a snapshot; the count beside them is live from the Tickets sheet.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I38"/>
+  <autoFilter ref="A4:I37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>